<commit_message>
Field Picarro calibration added
Added Excel sheet of the field Picarro calibration done in December

Sheet was created by Flavia Pierre
</commit_message>
<xml_diff>
--- a/Field-trails/Picarro-Calibration-2025-12-05-field-picarro.xlsx
+++ b/Field-trails/Picarro-Calibration-2025-12-05-field-picarro.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F1C34D1-6240-4CB9-81F4-C657C409D0CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75EE0AA7-FAEC-4528-8805-E9380C8B6DF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,15 +32,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="18">
   <si>
     <t>Air flow</t>
   </si>
   <si>
     <t>NH3 Flow</t>
-  </si>
-  <si>
-    <t>Expected concentration</t>
   </si>
   <si>
     <t>Measured Concentration</t>
@@ -80,6 +77,15 @@
   </si>
   <si>
     <t>Time (hh:mm) PICARRO</t>
+  </si>
+  <si>
+    <t>C Nh3 cylinder (ppb)</t>
+  </si>
+  <si>
+    <t>Expected concentration -theoretical cylinder c</t>
+  </si>
+  <si>
+    <t>Expected - measured cylinder c</t>
   </si>
 </sst>
 </file>
@@ -395,7 +401,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'Sheet1 (2)'!$F$3:$F$9</c:f>
+              <c:f>'Sheet1 (2)'!$G$3:$G$9</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="7"/>
@@ -878,34 +884,37 @@
           </c:trendline>
           <c:xVal>
             <c:numRef>
-              <c:f>'Sheet1 (2)'!$E$3:$E$8</c:f>
+              <c:f>'Sheet1 (2)'!$F$3:$F$9</c:f>
               <c:numCache>
-                <c:formatCode>0.0</c:formatCode>
-                <c:ptCount val="6"/>
+                <c:formatCode>0.00</c:formatCode>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>243.90243902439028</c:v>
+                  <c:v>217.5606341463415</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>697.67441860465124</c:v>
+                  <c:v>622.32460465116287</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1011.2359550561797</c:v>
+                  <c:v>902.02105617977531</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1578.9473684210527</c:v>
+                  <c:v>1408.4188421052634</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>2000</c:v>
+                  <c:v>1783.9972000000002</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>8919.9860000000008</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'Sheet1 (2)'!$F$3:$F$8</c:f>
+              <c:f>'Sheet1 (2)'!$G$3:$G$8</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="6"/>
@@ -1029,7 +1038,7 @@
             </a:p>
           </c:txPr>
         </c:title>
-        <c:numFmt formatCode="0.0" sourceLinked="1"/>
+        <c:numFmt formatCode="0.00" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -2361,15 +2370,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>1385101</xdr:colOff>
-      <xdr:row>12</xdr:row>
-      <xdr:rowOff>90852</xdr:rowOff>
+      <xdr:colOff>1526212</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>175519</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>227146</xdr:colOff>
-      <xdr:row>25</xdr:row>
-      <xdr:rowOff>24843</xdr:rowOff>
+      <xdr:colOff>368257</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>109510</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -2399,15 +2408,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>1251184</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>47037</xdr:rowOff>
+      <xdr:colOff>1580444</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>65852</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>93229</xdr:colOff>
-      <xdr:row>38</xdr:row>
-      <xdr:rowOff>159769</xdr:rowOff>
+      <xdr:colOff>422489</xdr:colOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>178584</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -2754,16 +2763,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{50826081-2711-4C45-BA43-CD7F10063201}">
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr defaultColWidth="17.33203125" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="20" customWidth="1"/>
     <col min="4" max="4" width="19.33203125" customWidth="1"/>
-    <col min="5" max="5" width="20.21875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="40.109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="42.21875" customWidth="1"/>
+    <col min="7" max="7" width="22.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
@@ -2773,78 +2783,88 @@
       </c>
       <c r="D1" s="20"/>
       <c r="E1" t="s">
+        <v>16</v>
+      </c>
+      <c r="F1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1" t="s">
         <v>2</v>
       </c>
-      <c r="F1" t="s">
+      <c r="H1" s="21" t="s">
+        <v>14</v>
+      </c>
+      <c r="I1" s="21"/>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="21" t="s">
-        <v>15</v>
-      </c>
-      <c r="H1" s="21"/>
+      <c r="B2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I2" t="s">
+        <v>8</v>
+      </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E2" t="s">
-        <v>7</v>
-      </c>
-      <c r="F2" t="s">
-        <v>7</v>
-      </c>
-      <c r="G2" t="s">
-        <v>8</v>
-      </c>
-      <c r="H2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B3" s="8">
         <v>4</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D3" s="10">
         <v>0</v>
       </c>
       <c r="E3" s="7">
-        <f t="shared" ref="E3:E9" si="0">+$E$12*D3/(B3+D3)</f>
+        <f>+$E$12*D3/(B3+D3)</f>
         <v>0</v>
       </c>
       <c r="F3" s="3">
+        <f>($E$13*D3)/(B3+D3)</f>
+        <v>0</v>
+      </c>
+      <c r="G3" s="3">
         <v>1.2210000000000001</v>
       </c>
-      <c r="G3" s="4">
+      <c r="H3" s="4">
         <v>0.37152777777777779</v>
       </c>
-      <c r="H3" s="4">
+      <c r="I3" s="4">
         <v>0.38194444444444442</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B4" s="8">
         <v>4</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D4" s="10">
         <v>0.1</v>
@@ -2854,180 +2874,211 @@
         <v>243.90243902439028</v>
       </c>
       <c r="F4" s="3">
+        <f t="shared" ref="F4:F9" si="0">($E$13*D4)/(B4+D4)</f>
+        <v>217.5606341463415</v>
+      </c>
+      <c r="G4" s="3">
         <v>244.70400000000001</v>
       </c>
-      <c r="G4" s="4">
+      <c r="H4" s="4">
         <v>0.4513888888888889</v>
       </c>
-      <c r="H4" s="18">
+      <c r="I4" s="18">
         <v>0.46180555555555558</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B5" s="8">
         <v>4</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D5" s="10">
         <v>0.3</v>
       </c>
       <c r="E5" s="7">
+        <f t="shared" ref="E3:E9" si="1">+$E$12*D5/(B5+D5)</f>
+        <v>697.67441860465124</v>
+      </c>
+      <c r="F5" s="3">
         <f t="shared" si="0"/>
-        <v>697.67441860465124</v>
-      </c>
-      <c r="F5" s="3">
+        <v>622.32460465116287</v>
+      </c>
+      <c r="G5" s="3">
         <v>665.30799999999999</v>
       </c>
-      <c r="G5" s="4">
+      <c r="H5" s="4">
         <v>0.44097222222222221</v>
       </c>
-      <c r="H5" s="4">
+      <c r="I5" s="4">
         <v>0.4513888888888889</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="13" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B6" s="14">
         <v>4</v>
       </c>
       <c r="C6" s="15" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D6" s="16">
         <v>0.45</v>
       </c>
       <c r="E6" s="7">
+        <f t="shared" si="1"/>
+        <v>1011.2359550561797</v>
+      </c>
+      <c r="F6" s="3">
         <f t="shared" si="0"/>
-        <v>1011.2359550561797</v>
-      </c>
-      <c r="F6" s="3">
+        <v>902.02105617977531</v>
+      </c>
+      <c r="G6" s="3">
         <v>951.33399999999995</v>
       </c>
-      <c r="G6" s="4">
+      <c r="H6" s="4">
         <v>0.42916666666666664</v>
       </c>
-      <c r="H6" s="4">
+      <c r="I6" s="4">
         <v>0.44097222222222221</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B7" s="8">
         <v>4</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D7" s="10">
         <v>0.75</v>
       </c>
       <c r="E7" s="7">
+        <f t="shared" si="1"/>
+        <v>1578.9473684210527</v>
+      </c>
+      <c r="F7" s="3">
         <f t="shared" si="0"/>
-        <v>1578.9473684210527</v>
-      </c>
-      <c r="F7" s="3">
+        <v>1408.4188421052634</v>
+      </c>
+      <c r="G7" s="3">
         <v>1480.23</v>
       </c>
-      <c r="G7" s="4">
+      <c r="H7" s="4">
         <v>0.40625</v>
       </c>
-      <c r="H7" s="4">
+      <c r="I7" s="4">
         <v>0.41666666666666669</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B8" s="8">
         <v>4</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D8" s="10">
         <v>1</v>
       </c>
       <c r="E8" s="7">
+        <f t="shared" si="1"/>
+        <v>2000</v>
+      </c>
+      <c r="F8" s="3">
         <f t="shared" si="0"/>
-        <v>2000</v>
-      </c>
-      <c r="F8" s="3">
+        <v>1783.9972000000002</v>
+      </c>
+      <c r="G8" s="3">
         <v>1841.5419999999999</v>
       </c>
-      <c r="G8" s="4">
+      <c r="H8" s="4">
         <v>0.38750000000000001</v>
       </c>
-      <c r="H8" s="12">
+      <c r="I8" s="12">
         <v>0.40625</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B9" s="10">
         <v>0</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D9" s="8">
         <v>4</v>
       </c>
       <c r="E9" s="7">
+        <f t="shared" si="1"/>
+        <v>10000</v>
+      </c>
+      <c r="F9" s="3">
         <f t="shared" si="0"/>
-        <v>10000</v>
-      </c>
-      <c r="F9" s="3">
         <v>8919.9860000000008</v>
       </c>
-      <c r="G9" s="4">
+      <c r="G9" s="3">
+        <v>8919.9860000000008</v>
+      </c>
+      <c r="H9" s="4">
         <v>0.46875</v>
       </c>
-      <c r="H9" s="4">
+      <c r="I9" s="4">
         <v>0.47916666666666669</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="G10" s="4"/>
       <c r="H10" s="4"/>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B11" s="9" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" s="5"/>
       <c r="B12" s="11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C12" s="5">
         <v>1</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E12" s="6">
         <v>10000</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C13">
         <f>+C12*0.1</f>
         <v>0.1</v>
+      </c>
+      <c r="D13" t="s">
+        <v>15</v>
+      </c>
+      <c r="E13" s="3">
+        <f>G9</f>
+        <v>8919.9860000000008</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
@@ -3053,7 +3104,7 @@
   <mergeCells count="3">
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C1:D1"/>
-    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="H1:I1"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3072,21 +3123,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<TemplafyFormConfiguration><![CDATA[{"formFields":[],"formDataEntries":[]}]]></TemplafyFormConfiguration>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <TemplafyTemplateConfiguration><![CDATA[{"transformationConfigurations":[],"templateName":"blankspreadsheet","templateDescription":"","enableDocumentContentUpdater":false,"version":"2.0"}]]></TemplafyTemplateConfiguration>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<TemplafyFormConfiguration><![CDATA[{"formFields":[],"formDataEntries":[]}]]></TemplafyFormConfiguration>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7408D0D6-C97A-426B-8466-DDDAA7A3F420}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{613AEFFE-C095-42A7-A0AC-5564FFC1D197}">
   <ds:schemaRefs/>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{613AEFFE-C095-42A7-A0AC-5564FFC1D197}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7408D0D6-C97A-426B-8466-DDDAA7A3F420}">
   <ds:schemaRefs/>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
started on Merge function
Started on function to merge triplicates
specifically backgrunds such that averaged bkg flux can be subtracted before downstream integration
</commit_message>
<xml_diff>
--- a/Field-trails/Picarro-Calibration-2025-12-05-field-picarro.xlsx
+++ b/Field-trails/Picarro-Calibration-2025-12-05-field-picarro.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75EE0AA7-FAEC-4528-8805-E9380C8B6DF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4029C68D-96A3-43DE-87EE-6A0DA06EF845}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -758,6 +758,36 @@
   </mc:AlternateContent>
   <c:chart>
     <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="da-DK"/>
+              <a:t>Forced</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="da-DK" baseline="0"/>
+              <a:t> intercept 10,000 pt removed</a:t>
+            </a:r>
+            <a:endParaRPr lang="da-DK"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -843,13 +873,43 @@
               <a:effectLst/>
             </c:spPr>
             <c:trendlineType val="linear"/>
+            <c:dispRSqr val="0"/>
+            <c:dispEq val="0"/>
+          </c:trendline>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="linear"/>
+            <c:intercept val="0"/>
+            <c:dispRSqr val="0"/>
+            <c:dispEq val="0"/>
+          </c:trendline>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="linear"/>
+            <c:intercept val="0"/>
             <c:dispRSqr val="1"/>
             <c:dispEq val="1"/>
             <c:trendlineLbl>
               <c:layout>
                 <c:manualLayout>
-                  <c:x val="0.12345174323103394"/>
-                  <c:y val="0.26951246466966777"/>
+                  <c:x val="1.0438117659448745E-3"/>
+                  <c:y val="-0.20302034752511605"/>
                 </c:manualLayout>
               </c:layout>
               <c:numFmt formatCode="General" sourceLinked="0"/>
@@ -877,7 +937,7 @@
                       <a:cs typeface="+mn-cs"/>
                     </a:defRPr>
                   </a:pPr>
-                  <a:endParaRPr lang="en-DK"/>
+                  <a:endParaRPr lang="da-DK"/>
                 </a:p>
               </c:txPr>
             </c:trendlineLbl>
@@ -2901,7 +2961,7 @@
         <v>0.3</v>
       </c>
       <c r="E5" s="7">
-        <f t="shared" ref="E3:E9" si="1">+$E$12*D5/(B5+D5)</f>
+        <f t="shared" ref="E5:E9" si="1">+$E$12*D5/(B5+D5)</f>
         <v>697.67441860465124</v>
       </c>
       <c r="F5" s="3">

</xml_diff>